<commit_message>
Chon Che do, Chuong trinh lam gi
</commit_message>
<xml_diff>
--- a/Sosanh_code_thucte.xlsx
+++ b/Sosanh_code_thucte.xlsx
@@ -5,15 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Github\longhoney\ledGT-Long-kxnTask\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Arduino\Uno_Sketch\ledGT-Long-kxnTask\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8A44E1-5247-423B-BB27-F58F672AF276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF9A46C-6BC0-4B26-A5E8-8DA5E397728A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="CheDo" sheetId="2" r:id="rId2"/>
+    <sheet name="DanY-Ham" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="116">
   <si>
     <t>Đèn giao thông</t>
   </si>
@@ -1305,13 +1307,709 @@
       </rPr>
       <t>()</t>
     </r>
+  </si>
+  <si>
+    <t>Mô tả nhanh</t>
+  </si>
+  <si>
+    <t>ledGT_kxnTask.ino</t>
+  </si>
+  <si>
+    <t>Chương trình điều khiển chính</t>
+  </si>
+  <si>
+    <t>khoiApp.h</t>
+  </si>
+  <si>
+    <t>Chứa Dữ liệu: đối tượng được điều khiển, khai báo chân, khai báo thời gian sáng đèn</t>
+  </si>
+  <si>
+    <t>Chạy chương trình quản lý các chế độ hoạt động</t>
+  </si>
+  <si>
+    <t>Thực hiện các công việc trong chế độ hoạt động</t>
+  </si>
+  <si>
+    <t>khoiGT.h</t>
+  </si>
+  <si>
+    <t>Lưu Chế độ sáng luân phiên 3 đèn: Đỏ - Xanh - Vàng và Chế độ Tắt cả 3 đèn</t>
+  </si>
+  <si>
+    <t>khoiBlink.h</t>
+  </si>
+  <si>
+    <t>Lưu Chế độ Sáng/tắt đèn Vàng mỗi X giây</t>
+  </si>
+  <si>
+    <t>Quy định thứ tự thực hiện công việc của chế độ: thứ tự sáng đèn, thời gian sáng đèn, khai báo chân</t>
+  </si>
+  <si>
+    <t>Mô tả các bước nhỏ trong công việc: sáng/tắt đèn, định nghĩ trạng thái làm việc …</t>
+  </si>
+  <si>
+    <t>Nhận lệnh từ người dùng: Bấm số 0 thì tắt đèn, bấm số 2 thì sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <t>Chương trình quản lý, dùng thư viện kxnTaskManager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cấp </t>
+  </si>
+  <si>
+    <t>3a</t>
+  </si>
+  <si>
+    <t>3b</t>
+  </si>
+  <si>
+    <t>Chế độ/ Chương trình</t>
+  </si>
+  <si>
+    <r>
+      <t>khoiApp1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>stop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF728E00"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> '0':</t>
+    </r>
+  </si>
+  <si>
+    <t>Chọn Chế độ 0: tắt 3 đèn</t>
+  </si>
+  <si>
+    <r>
+      <t>khoiGT1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>stop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>khoiBlinkY1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>stop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>Tại hàm stop(), ngưng Chế độ sáng luân phiên 3 đèn và ngưng Chế độ sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <t>Tại hàm stop(), tắt các đèn = đặt các chân tín hiệu xuống mức Thấp</t>
+  </si>
+  <si>
+    <t>Tại hàm stop(), tắt  đèn = đặt  chân tín hiệu xuống mức Thấp</t>
+  </si>
+  <si>
+    <t>Sáng luân phiên 3 đèn: Đỏ - Xanh - Vàng</t>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> '3':</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>khoiApp1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>startThreeColor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>Chọn Chế độ 3: Sáng luân phiên 3 đèn</t>
+  </si>
+  <si>
+    <r>
+      <t>khoiGT1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>startR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> khoiGT_ON_R:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>digitalWrite</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">pinR, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF005C5F"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>Ngưng Chế độ sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <t>Tại case sáng đèn xanh, đặt chân đèn xanh mức Cao và đặt 2 chân đèn còn lại mức Thấp</t>
+  </si>
+  <si>
+    <t>Sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <r>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF728E00"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> '2':</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>khoiApp1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>startBlinkYellow-Color</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>khoiBlinkY1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>digitalWrite</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>pinY, 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> khoiBlink_ON:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> khoiBlink_OFF:</t>
+    </r>
+  </si>
+  <si>
+    <t>Lặp lại ở 2 case còn lại</t>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> khoiGT_ON_G:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>case</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> khoiGT_ON_Y:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FFD35400"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>digitalWrite</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">pinR, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF005C5F"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF434F54"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF4E5B61"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>Tại case sáng đèn, đặt chân đèn mức Cao và ngược lại</t>
+  </si>
+  <si>
+    <t>Ngưng chế độ sáng 3 đèn luân phiên</t>
+  </si>
+  <si>
+    <t>Thực hiện công việc sáng đèn xanh, sau đó luân phiên với 2 đèn còn lại</t>
+  </si>
+  <si>
+    <t>(Tôi chưa hiểu tại sao lại đặt là startR)</t>
+  </si>
+  <si>
+    <t>Thực hiện chế độ sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <t>Chọn chế độ sáng/tắt đèn vàng</t>
+  </si>
+  <si>
+    <t>Mỗi 1 hàm đều có cấu trúc cơ bản:</t>
+  </si>
+  <si>
+    <t>Thêm vào chương trình quản lý</t>
+  </si>
+  <si>
+    <t>Đặt thành chế độ (Abc)</t>
+  </si>
+  <si>
+    <t>Nội dung thực hiện</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1380,13 +2078,39 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF728E00"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="16">
@@ -1570,7 +2294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1622,6 +2346,182 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1903,19 +2803,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W32"/>
-  <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="25"/>
-    <col min="2" max="6" width="9.140625" style="1"/>
-    <col min="7" max="7" width="9.140625" style="25"/>
-    <col min="8" max="12" width="9.140625" style="1"/>
-    <col min="13" max="13" width="9.140625" style="7"/>
-    <col min="14" max="14" width="9.140625" style="12"/>
-    <col min="15" max="15" width="9.140625" style="7"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.1796875" style="25"/>
+    <col min="2" max="6" width="9.1796875" style="1"/>
+    <col min="7" max="7" width="9.1796875" style="25"/>
+    <col min="8" max="12" width="9.1796875" style="1"/>
+    <col min="13" max="13" width="9.1796875" style="7"/>
+    <col min="14" max="14" width="9.1796875" style="12"/>
+    <col min="15" max="15" width="9.1796875" style="7"/>
+    <col min="16" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -1924,7 +2824,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
@@ -1958,7 +2858,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="24">
         <v>2</v>
       </c>
@@ -1989,7 +2889,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G4" s="27"/>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -2004,7 +2904,7 @@
       <c r="Q4" s="16"/>
       <c r="R4" s="18"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="26">
         <v>2</v>
       </c>
@@ -2023,7 +2923,7 @@
       <c r="Q5" s="20"/>
       <c r="R5" s="22"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G6" s="24">
         <v>3</v>
       </c>
@@ -2044,7 +2944,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G7" s="27"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -2059,7 +2959,7 @@
       <c r="Q7" s="16"/>
       <c r="R7" s="18"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="26">
         <v>4</v>
       </c>
@@ -2079,7 +2979,7 @@
       <c r="Q8" s="20"/>
       <c r="R8" s="22"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" s="24">
         <v>3</v>
       </c>
@@ -2117,7 +3017,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -2135,7 +3035,7 @@
       <c r="Q10" s="12"/>
       <c r="R10" s="14"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -2153,7 +3053,7 @@
       <c r="Q11" s="12"/>
       <c r="R11" s="14"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -2172,7 +3072,7 @@
       <c r="Q12" s="16"/>
       <c r="R12" s="18"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -2196,7 +3096,7 @@
       <c r="Q13" s="20"/>
       <c r="R13" s="22"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
@@ -2225,7 +3125,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B15" s="12"/>
       <c r="C15" s="16"/>
       <c r="D15" s="12"/>
@@ -2243,7 +3143,7 @@
       <c r="Q15" s="12"/>
       <c r="R15" s="14"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.4">
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -2261,7 +3161,7 @@
       <c r="Q16" s="12"/>
       <c r="R16" s="14"/>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -2280,7 +3180,7 @@
       <c r="Q17" s="16"/>
       <c r="R17" s="18"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -2304,7 +3204,7 @@
       <c r="Q18" s="20"/>
       <c r="R18" s="22"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -2334,7 +3234,7 @@
       </c>
       <c r="W19" s="12"/>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -2353,7 +3253,7 @@
       <c r="R20" s="14"/>
       <c r="W20" s="12"/>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -2371,7 +3271,7 @@
       <c r="Q21" s="12"/>
       <c r="R21" s="14"/>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
@@ -2391,7 +3291,7 @@
       <c r="Q22" s="16"/>
       <c r="R22" s="18"/>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
@@ -2415,7 +3315,7 @@
       <c r="Q23" s="20"/>
       <c r="R23" s="22"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
@@ -2439,7 +3339,7 @@
       <c r="Q24" s="20"/>
       <c r="R24" s="22"/>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A25" s="24">
         <v>0</v>
       </c>
@@ -2471,7 +3371,7 @@
       <c r="Q25" s="9"/>
       <c r="R25" s="11"/>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
@@ -2489,7 +3389,7 @@
       <c r="Q26" s="12"/>
       <c r="R26" s="14"/>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
@@ -2507,7 +3407,7 @@
       <c r="Q27" s="12"/>
       <c r="R27" s="14"/>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B28" s="12"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
@@ -2526,7 +3426,7 @@
       <c r="Q28" s="16"/>
       <c r="R28" s="18"/>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.4">
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
@@ -2551,15 +3451,1036 @@
       <c r="Q29" s="20"/>
       <c r="R29" s="22"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.4">
       <c r="P30" s="12"/>
       <c r="Q30" s="12"/>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.4">
       <c r="Q31" s="24"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.4">
       <c r="Q32" s="27"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECD18DB9-CCF7-45A9-954E-462E4E8B5E49}">
+  <dimension ref="A1:S39"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A1" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="36">
+        <v>1</v>
+      </c>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="36">
+        <v>2</v>
+      </c>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="38"/>
+      <c r="P1" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="38"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A2" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="49" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q2" s="39"/>
+      <c r="R2" s="39"/>
+      <c r="S2" s="40"/>
+    </row>
+    <row r="3" spans="1:19" ht="70" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="50" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" s="51"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="52"/>
+      <c r="P3" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q3" s="51"/>
+      <c r="R3" s="51"/>
+      <c r="S3" s="52"/>
+    </row>
+    <row r="4" spans="1:19" ht="78.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="50" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="51"/>
+      <c r="F4" s="51"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="51"/>
+      <c r="J4" s="51"/>
+      <c r="K4" s="52"/>
+      <c r="L4" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" s="51"/>
+      <c r="N4" s="51"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q4" s="51"/>
+      <c r="R4" s="51"/>
+      <c r="S4" s="52"/>
+    </row>
+    <row r="5" spans="1:19" ht="78.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="46"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="50" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="M5" s="51"/>
+      <c r="N5" s="51"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="50" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q5" s="51"/>
+      <c r="R5" s="51"/>
+      <c r="S5" s="52"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A8" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="34"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="34"/>
+      <c r="P8" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q8" s="34"/>
+      <c r="R8" s="34"/>
+      <c r="S8" s="34"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A9" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="54"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="72" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="11"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A10" s="55"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="73" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="14"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A11" s="55"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="S11" s="18"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A12" s="55"/>
+      <c r="B12" s="56"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="74" t="s">
+        <v>82</v>
+      </c>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="74"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="74" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="18"/>
+    </row>
+    <row r="13" spans="1:19" ht="64" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="58"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="75" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="75"/>
+      <c r="F13" s="75"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="M13" s="30"/>
+      <c r="N13" s="30"/>
+      <c r="O13" s="30"/>
+      <c r="P13" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q13" s="30"/>
+      <c r="R13" s="30"/>
+      <c r="S13" s="30"/>
+    </row>
+    <row r="14" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="62"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="76" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="76" t="s">
+        <v>91</v>
+      </c>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="76"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="S14" s="11"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A15" s="64"/>
+      <c r="B15" s="65"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="73" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="73" t="s">
+        <v>92</v>
+      </c>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="73"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="14"/>
+    </row>
+    <row r="16" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="64"/>
+      <c r="B16" s="65"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="79" t="s">
+        <v>109</v>
+      </c>
+      <c r="I16" s="80"/>
+      <c r="J16" s="80"/>
+      <c r="K16" s="81"/>
+      <c r="L16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="14"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A17" s="64"/>
+      <c r="B17" s="65"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="79"/>
+      <c r="I17" s="80"/>
+      <c r="J17" s="80"/>
+      <c r="K17" s="81"/>
+      <c r="L17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="14"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A18" s="64"/>
+      <c r="B18" s="65"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="14"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A19" s="64"/>
+      <c r="B19" s="65"/>
+      <c r="C19" s="66"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="78" t="s">
+        <v>103</v>
+      </c>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+      <c r="S19" s="14"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A20" s="64"/>
+      <c r="B20" s="65"/>
+      <c r="C20" s="66"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="14"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A21" s="64"/>
+      <c r="B21" s="65"/>
+      <c r="C21" s="66"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="14"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A22" s="64"/>
+      <c r="B22" s="65"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="14"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A23" s="64"/>
+      <c r="B23" s="65"/>
+      <c r="C23" s="66"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="14"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="14"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A24" s="64"/>
+      <c r="B24" s="65"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="78" t="s">
+        <v>104</v>
+      </c>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="7"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="14"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A25" s="64"/>
+      <c r="B25" s="65"/>
+      <c r="C25" s="66"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="14"/>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="14"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A26" s="64"/>
+      <c r="B26" s="65"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="14"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="14"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A27" s="64"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="74" t="s">
+        <v>24</v>
+      </c>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="15"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="18"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A28" s="64"/>
+      <c r="B28" s="65"/>
+      <c r="C28" s="66"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="18"/>
+    </row>
+    <row r="29" spans="1:19" ht="64.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="64"/>
+      <c r="B29" s="65"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="70"/>
+      <c r="H29" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="I29" s="62"/>
+      <c r="J29" s="62"/>
+      <c r="K29" s="70"/>
+      <c r="L29" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="M29" s="62"/>
+      <c r="N29" s="62"/>
+      <c r="O29" s="70"/>
+      <c r="P29" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q29" s="62"/>
+      <c r="R29" s="62"/>
+      <c r="S29" s="70"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A30" s="67"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="71"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="M30" s="31"/>
+      <c r="N30" s="31"/>
+      <c r="O30" s="33"/>
+      <c r="P30" s="15"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="18"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A31" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="62"/>
+      <c r="C31" s="70"/>
+      <c r="D31" s="72" t="s">
+        <v>96</v>
+      </c>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="11"/>
+      <c r="L31" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9"/>
+      <c r="O31" s="11"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
+      <c r="S31" s="11"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A32" s="64"/>
+      <c r="B32" s="65"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="85" t="s">
+        <v>97</v>
+      </c>
+      <c r="E32" s="86"/>
+      <c r="F32" s="86"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="14"/>
+      <c r="P32" s="7"/>
+      <c r="Q32" s="12"/>
+      <c r="R32" s="12"/>
+      <c r="S32" s="14"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A33" s="64"/>
+      <c r="B33" s="65"/>
+      <c r="C33" s="66"/>
+      <c r="D33" s="85"/>
+      <c r="E33" s="86"/>
+      <c r="F33" s="86"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="M33" s="16"/>
+      <c r="N33" s="16"/>
+      <c r="O33" s="18"/>
+      <c r="P33" s="15"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="S33" s="18"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A34" s="64"/>
+      <c r="B34" s="65"/>
+      <c r="C34" s="66"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="11"/>
+      <c r="P34" s="76" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="11"/>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A35" s="64"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="66"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="14"/>
+      <c r="P35" s="88" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="14"/>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A36" s="64"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="66"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="14"/>
+      <c r="P36" s="78" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q36" s="12"/>
+      <c r="R36" s="12"/>
+      <c r="S36" s="14"/>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A37" s="64"/>
+      <c r="B37" s="65"/>
+      <c r="C37" s="66"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="18"/>
+      <c r="P37" s="77" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="18"/>
+    </row>
+    <row r="38" spans="1:19" ht="51.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="64"/>
+      <c r="B38" s="65"/>
+      <c r="C38" s="66"/>
+      <c r="D38" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="E38" s="54"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="68"/>
+      <c r="H38" s="82" t="s">
+        <v>107</v>
+      </c>
+      <c r="I38" s="83"/>
+      <c r="J38" s="83"/>
+      <c r="K38" s="83"/>
+      <c r="L38" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="M38" s="62"/>
+      <c r="N38" s="62"/>
+      <c r="O38" s="70"/>
+      <c r="P38" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q38" s="83"/>
+      <c r="R38" s="83"/>
+      <c r="S38" s="84"/>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A39" s="67"/>
+      <c r="B39" s="60"/>
+      <c r="C39" s="71"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="I39" s="31"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="15"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="15"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
+      <c r="S39" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="47">
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="A31:C39"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="H29:K29"/>
+    <mergeCell ref="D32:G33"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L30:O30"/>
+    <mergeCell ref="H16:K17"/>
+    <mergeCell ref="H38:K38"/>
+    <mergeCell ref="P38:S38"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="A9:C13"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="P8:S8"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="L29:O29"/>
+    <mergeCell ref="P29:S29"/>
+    <mergeCell ref="H30:K30"/>
+    <mergeCell ref="A14:C30"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C5"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="P3:S3"/>
+    <mergeCell ref="P4:S4"/>
+    <mergeCell ref="P5:S5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3286853A-7D55-47CC-9F61-860794F3EBB0}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>114</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>